<commit_message>
Update approved jobs sheet
</commit_message>
<xml_diff>
--- a/approved_jobs.xlsx
+++ b/approved_jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -471,55 +471,55 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-22T12:33:35.076089+00:00</t>
+          <t>2026-08-25T14:24:51.17624+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Backend Intern</t>
+          <t>Product Operations Intern</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Smallcase</t>
+          <t>Fampay</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://app.pyjamahr.com/careers?company=smallcase&amp;job_id=256252&amp;company_uuid=2615584222</t>
+          <t>https://jobs.lever.co/fampay/e21b862f-cde6-4fb7-a08b-02c72f26ae99</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
+          <t>About Fam (previously FamPay) Fam is India’s first payments app for everyone above 11. FamApp helps make online and offline payments through UPI and FamCard. We are on a mission to raise a new, financially aware generation, and drive 250 million+ young users in India to kickstart their financial journey super early in their life. We’re reimagining how the next generation experiences fintech—going beyond payments to build a lifestyle brand that blends money, identity, and everyday experiences into one seamless, intuitive journey. Founded in 2019 by IIT Roorkee alumni, Fam is backed by some of the most respected investors around the world like Elevation Capital, Y-Combinator, Peak XV (Sequoia Capital) India, Venture Highway, Global Founder’s Capital and the likes of Kunal Shah, Amrish Rao as angel investors. About this role This role is operations heavy role with analytics as an added responsibility. You need to be comfortable executing campaigns relentlessly and working with data. You’ll be majorly working on Category Growth projects and Product Operations along with delivering high-quality outcomes in a fast-paced, dynamic environment. Understand that outcomes &gt; outputs</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-22T12:33:32.004558+00:00</t>
+          <t>2026-08-25T14:24:11.044632+00:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Meritshot</t>
+          <t>Enterpret</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -531,7 +531,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4454242112/</t>
+          <t>https://job-boards.greenhouse.io/enterpret/jobs/7847134003</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -543,12 +543,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-22T12:33:28.837146+00:00</t>
+          <t>2026-08-25T14:24:07.705529+00:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -558,18 +558,18 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Remote (Work From Home)</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://bit.ly/4qkLIuH</t>
+          <t>https://bit.ly/45LFHxK</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -581,33 +581,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-22T12:33:26.419583+00:00</t>
+          <t>2026-08-25T14:24:05.267553+00:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Remote (Work From Home)</t>
+          <t>Bengaluru/Hyderabad/Delhi/Pune/Chennai</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://bit.ly/45nkUAn</t>
+          <t>https://www.amazon.jobs/en/jobs/10506481/sde-i-intern-amazon-university-talent-acquisition</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -619,12 +619,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-22T12:33:20.104134+00:00</t>
+          <t>2026-08-25T14:23:37.191168+00:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AI Facial Data Collection Contributor</t>
+          <t>MCP Expert</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://bit.ly/4gbo4vO</t>
+          <t>https://bit.ly/4wJiMOk</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -657,17 +657,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-22T12:33:05.251094+00:00</t>
+          <t>2026-08-25T14:23:33.82492+00:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Software Engineering Intern (Summer)</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -679,7 +679,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.salesforce.com/company/careers/jobs/JR337715/summer-2027-intern-software-engineer/</t>
+          <t>https://careers.hpe.com/us/en/job/1211844/Intern</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -691,89 +691,93 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-22T12:33:03.503245+00:00</t>
+          <t>2026-08-25T14:23:25.612917+00:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Backend Java Developer</t>
+          <t>DevOps Engineering Intern</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>Fampay</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Remote (Work From Home)</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://bit.ly/4wRJpkA</t>
+          <t>https://jobs.lever.co/fampay/293a18f9-446a-437c-ba5d-d1300094b833</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
+          <t xml:space="preserve">About Fam (previously FamPay) Fam is India’s first payments app for everyone above 11. FamApp helps make online and offline payments through UPI and FamCard. We are on a mission to raise a new, financially aware generation, and drive 250 million+ young users in India to kickstart their financial journey super early in their life. We’re reimagining how the next generation experiences fintech—going beyond payments to build a lifestyle brand that blends money, identity, and everyday experiences into one seamless, intuitive journey. Founded in 2019 by IIT Roorkee alumni, Fam is backed by some of the most respected investors around the world like Elevation Capital, Y-Combinator, Peak XV (Sequoia Capital) India, Venture Highway, Global Founder’s Capital and the likes of Kunal Shah, Amrish Rao as angel investors. About this Role Always ready for with a Plan C because Plan A and B didn't work? We are looking for you! We’re looking for builders who enjoy creating things from scratch, breaking them, figuring out why they broke, and making them better. As a DevOps Engineer at FamApp, you’ll work at the intersection of infrastructure, reliability, and DevEx. You’ll help build the systems that </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-22T12:33:01.650538+00:00</t>
+          <t>2026-08-25T14:22:34.800573+00:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data Analyst Intern</t>
+          <t>DevOps Intern</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SWIFT</t>
+          <t>Cloudsek</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://goswift.keka.com/careers/jobdetails/153432</t>
+          <t>https://job-boards.greenhouse.io/cloudsek/jobs/6149788004</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
+          <t>DevOps Intern</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:59.807222+00:00</t>
+          <t>2026-08-25T14:22:23.10638+00:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NXP Semiconductor Women in Tech</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>NXP Semiconductors</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -782,10 +786,14 @@
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.nxp.com/company/about-nxp/events/women-in-tech:WOMEN-IN-TECH</t>
+          <t>https://bit.ly/45nkUAn</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -797,29 +805,33 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:56.748107+00:00</t>
+          <t>2026-08-25T14:22:21.002594+00:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FRND</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4455599485/</t>
+          <t>https://bit.ly/4qkLIuH</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -831,29 +843,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:54.751872+00:00</t>
+          <t>2026-08-25T14:22:16.887203+00:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Harman</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://jobsearch.harman.com/en_US/careers/searchjobs/R-54623-2026</t>
+          <t>https://bit.ly/4wZ8B9r</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -865,12 +881,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:52.811769+00:00</t>
+          <t>2026-08-25T14:22:13.458112+00:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AI Facial Data Collection Contributor</t>
+          <t>Fullstack Developer</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -880,18 +896,18 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>Full Stack</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Remote (Work From Home)</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://bit.ly/4hl4Ar1</t>
+          <t>https://bit.ly/3Sy7PRO</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -903,12 +919,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:50.619505+00:00</t>
+          <t>2026-08-25T14:22:10.397388+00:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>DevOps Engineer</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -924,12 +940,12 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Remote (Work From Home)</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://bit.ly/4hH3q9A</t>
+          <t>https://bit.ly/4gebHAv</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -941,33 +957,33 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:48.755864+00:00</t>
+          <t>2026-08-22T12:33:35.076089+00:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Software Engineer - AMTS</t>
+          <t>Backend Intern</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>Smallcase</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Hyderabad/Bangalore, India</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://bit.ly/4xGBIOS</t>
+          <t>https://app.pyjamahr.com/careers?company=smallcase&amp;job_id=256252&amp;company_uuid=2615584222</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -979,17 +995,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:46.368924+00:00</t>
+          <t>2026-08-22T12:33:32.004558+00:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Joveo</t>
+          <t>Meritshot</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1001,7 +1017,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4453427249/</t>
+          <t>https://www.linkedin.com/jobs/view/4454242112/</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1013,12 +1029,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:43.264285+00:00</t>
+          <t>2026-08-22T12:33:28.837146+00:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Fullstack Developer</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1028,7 +1044,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Full Stack</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -1039,7 +1055,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://bit.ly/3Sy7PRO</t>
+          <t>https://bit.ly/4qkLIuH</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1051,12 +1067,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:40.571545+00:00</t>
+          <t>2026-08-22T12:33:26.419583+00:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1066,7 +1082,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -1077,7 +1093,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://bit.ly/4wZ8B9r</t>
+          <t>https://bit.ly/45nkUAn</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1089,17 +1105,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-21T18:33:37.259219+00:00</t>
+          <t>2026-08-22T12:33:20.104134+00:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Intern - AI/ML</t>
+          <t>AI Facial Data Collection Contributor</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Towerresearchcapital</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1110,34 +1126,34 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>gurgaon</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8143756</t>
+          <t>https://bit.ly/4gbo4vO</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Intern - AI/ML</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-21T18:33:33.878834+00:00</t>
+          <t>2026-08-22T12:33:05.251094+00:00</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Quantitative Developer Intern</t>
+          <t>Software Engineering Intern (Summer)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Towerresearchcapital</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1146,324 +1162,320 @@
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8138524</t>
+          <t>https://www.salesforce.com/company/careers/jobs/JR337715/summer-2027-intern-software-engineer/</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Quantitative Developer Intern</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-21T18:33:29.313779+00:00</t>
+          <t>2026-08-22T12:33:03.503245+00:00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sales &amp; Customer Success Intern - EU</t>
+          <t>Backend Java Developer</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Truecaller</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Remote (Work From Home)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/truecaller/jobs/8138837</t>
+          <t>https://bit.ly/4wRJpkA</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Sales &amp; Customer Success Intern - EU</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-14T03:46:04.307219+00:00</t>
+          <t>2026-08-22T12:33:01.650538+00:00</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Quantitative Research Internship - 6 Months, Central Execution Research</t>
+          <t>Data Analyst Intern</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Towerresearchcapital</t>
+          <t>SWIFT</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8113986</t>
+          <t>https://goswift.keka.com/careers/jobdetails/153432</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Quantitative Research Internship - 6 Months, Central Execution Research</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-10T17:40:51.724814+00:00</t>
+          <t>2026-08-22T12:32:59.807222+00:00</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AI Engineer, Internship - Summer 2026 - Applications Open Now</t>
+          <t>NXP Semiconductor Women in Tech</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Postman</t>
+          <t>NXP Semiconductors</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Berkeley, California, United States; San Francisco, California, United States</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/postman/jobs/7823417003</t>
+          <t>https://www.nxp.com/company/about-nxp/events/women-in-tech:WOMEN-IN-TECH</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>AI Engineer, Internship - Summer 2026 - Applications Open Now</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-10T17:40:47.009978+00:00</t>
+          <t>2026-08-22T12:32:56.748107+00:00</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>[Backend] Software Engineering Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Enterpret</t>
+          <t>FRND</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Bengaluru, Onsite</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/enterpret/jobs/7847134003</t>
+          <t>https://www.linkedin.com/jobs/view/4455599485/</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>[Backend] Software Engineering Intern</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-08T04:12:52.37725+00:00</t>
+          <t>2026-08-22T12:32:54.751872+00:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Brand Marketing Intern</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Earnin</t>
+          <t>Harman</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/earnin/jobs/8113206</t>
+          <t>https://jobsearch.harman.com/en_US/careers/searchjobs/R-54623-2026</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Brand Marketing Intern</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-08T04:12:50.084908+00:00</t>
+          <t>2026-08-22T12:32:52.811769+00:00</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Customer Success Intern</t>
+          <t>AI Facial Data Collection Contributor</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Knowbe4</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Remote (Work From Home)</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/knowbe4/jobs/8660687002</t>
+          <t>https://bit.ly/4hl4Ar1</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Customer Success Intern</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-08T04:12:46.851447+00:00</t>
+          <t>2026-08-22T12:32:50.619505+00:00</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Product Marketing Intern - Tetriz</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Epifi</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Remote (Work From Home)</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/epifi/c6d070ce-d859-4d96-b82e-bca1fea37ddd</t>
+          <t>https://bit.ly/4hH3q9A</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Product Marketing Intern - Tetriz</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-08T04:12:45.117452+00:00</t>
+          <t>2026-08-22T12:32:48.755864+00:00</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Junior Execution Trader Intern</t>
+          <t>Software Engineer - AMTS</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Towerresearchcapital</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Hyderabad/Bangalore, India</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8091833</t>
+          <t>https://bit.ly/4xGBIOS</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Junior Execution Trader Intern</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:43.226773+00:00</t>
+          <t>2026-08-22T12:32:46.368924+00:00</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Copy Writer - Intern</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Joveo</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1475,131 +1487,143 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774341101</t>
+          <t>https://www.linkedin.com/jobs/view/4453427249/</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Copy Writer - Intern</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:36.983937+00:00</t>
+          <t>2026-08-22T12:32:43.264285+00:00</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Video Editor Intern</t>
+          <t>Fullstack Developer</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Full Stack</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Remote (Work From Home)</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4771440101</t>
+          <t>https://bit.ly/3Sy7PRO</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Video Editor Intern</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:35.138664+00:00</t>
+          <t>2026-08-22T12:32:40.571545+00:00</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Internship - Content </t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Remote (Work From Home)</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4819749101</t>
+          <t>https://bit.ly/4wZ8B9r</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Internship - Content</t>
+          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:33.590227+00:00</t>
+          <t>2026-08-21T18:33:37.259219+00:00</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Graphic Designer - Intern</t>
+          <t>Intern - AI/ML</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Towerresearchcapital</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>gurgaon</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774342101</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8143756</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Graphic Designer - Intern</t>
+          <t>Intern - AI/ML</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:31.543915+00:00</t>
+          <t>2026-08-21T18:33:33.878834+00:00</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Business Development Specialist (Outbound- International)</t>
+          <t>Quantitative Developer Intern</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Tide</t>
+          <t>Towerresearchcapital</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1608,32 +1632,36 @@
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/tide/jobs/7081017003</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8138524</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Business Development Specialist (Outbound- International)</t>
+          <t>Quantitative Developer Intern</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:28.879852+00:00</t>
+          <t>2026-08-21T18:33:29.313779+00:00</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Business Development Specialist (International Sales)</t>
+          <t>Sales &amp; Customer Success Intern - EU</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Tide</t>
+          <t>Truecaller</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1642,27 +1670,31 @@
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/tide/jobs/7598880003</t>
+          <t>https://job-boards.greenhouse.io/truecaller/jobs/8138837</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Business Development Specialist (International Sales)</t>
+          <t>Sales &amp; Customer Success Intern - EU</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:17.721593+00:00</t>
+          <t>2026-08-14T03:46:04.307219+00:00</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Risk Intern - 6 Month Internship Opportunity</t>
+          <t>Quantitative Research Internship - 6 Months, Central Execution Research</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1676,168 +1708,180 @@
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=7789933</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8113986</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Risk Intern - 6 Month Internship Opportunity</t>
+          <t>Quantitative Research Internship - 6 Months, Central Execution Research</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:10.248679+00:00</t>
+          <t>2026-08-10T17:40:51.724814+00:00</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Quantitative Trader Intern - Summer 2027</t>
+          <t>AI Engineer, Internship - Summer 2026 - Applications Open Now</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Towerresearchcapital</t>
+          <t>Postman</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Berkeley, California, United States; San Francisco, California, United States</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8024128</t>
+          <t>https://job-boards.greenhouse.io/postman/jobs/7823417003</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Quantitative Trader Intern - Summer 2027</t>
+          <t>AI Engineer, Internship - Summer 2026 - Applications Open Now</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:07.980596+00:00</t>
+          <t>2026-08-10T17:40:47.009978+00:00</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Quantitative Trader Intern, PhD</t>
+          <t>[Backend] Software Engineering Intern</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Towerresearchcapital</t>
+          <t>Enterpret</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Bengaluru, Onsite</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8024138</t>
+          <t>https://job-boards.greenhouse.io/enterpret/jobs/7847134003</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Quantitative Trader Intern, PhD</t>
+          <t>[Backend] Software Engineering Intern</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:05.838281+00:00</t>
+          <t>2026-08-08T04:12:52.37725+00:00</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Quantitative Developer Intern - Summer 2027</t>
+          <t>Brand Marketing Intern</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Towerresearchcapital</t>
+          <t>Earnin</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8044334</t>
+          <t>https://job-boards.greenhouse.io/earnin/jobs/8113206</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Quantitative Developer Intern - Summer 2027</t>
+          <t>Brand Marketing Intern</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:03.426202+00:00</t>
+          <t>2026-08-08T04:12:50.084908+00:00</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Business Analytics Intern - 6 Month Internship Opportunity</t>
+          <t>Customer Success Intern</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Towerresearchcapital</t>
+          <t>Knowbe4</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8041512</t>
+          <t>https://job-boards.greenhouse.io/knowbe4/jobs/8660687002</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Business Analytics Intern - 6 Month Internship Opportunity</t>
+          <t>Customer Success Intern</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:01.432263+00:00</t>
+          <t>2026-08-08T04:12:46.851447+00:00</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Sales Development Representative Intern (Hybrid)</t>
+          <t>Product Marketing Intern - Tetriz</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Knowbe4</t>
+          <t>Epifi</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1849,335 +1893,335 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/knowbe4/jobs/8566454002</t>
+          <t>https://jobs.lever.co/epifi/c6d070ce-d859-4d96-b82e-bca1fea37ddd</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Sales Development Representative Intern (Hybrid)</t>
+          <t>Product Marketing Intern - Tetriz</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:59.490728+00:00</t>
+          <t>2026-08-08T04:12:45.117452+00:00</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Sales Development Representative Intern (Hybrid)</t>
+          <t>Junior Execution Trader Intern</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Knowbe4</t>
+          <t>Towerresearchcapital</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/knowbe4/jobs/8566457002</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8091833</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Sales Development Representative Intern (Hybrid)</t>
+          <t>Junior Execution Trader Intern</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:55.183092+00:00</t>
+          <t>2026-07-27T16:30:43.226773+00:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Intern - Industrial Trainee</t>
+          <t>Copy Writer - Intern</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Inmobi</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/inmobi/jobs/8029868</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774341101</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Intern - Industrial Trainee</t>
+          <t>Copy Writer - Intern</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:52.581754+00:00</t>
+          <t>2026-07-27T16:30:36.983937+00:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Intern - Industrial Trainee</t>
+          <t>Video Editor Intern</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Inmobi</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/inmobi/jobs/7793050</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4771440101</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Intern - Industrial Trainee</t>
+          <t>Video Editor Intern</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:48.780995+00:00</t>
+          <t>2026-07-27T16:30:35.138664+00:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Security Consultant Intern</t>
+          <t xml:space="preserve">Internship - Content </t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Cloudsek</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/cloudsek/jobs/6115382004</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4819749101</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Security Consultant Intern</t>
+          <t>Internship - Content</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:47.193044+00:00</t>
+          <t>2026-07-27T16:30:33.590227+00:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">SDE Intern - Frontend   </t>
+          <t>Graphic Designer - Intern</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Cloudsek</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/cloudsek/jobs/5831215004</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774342101</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>SDE Intern - Frontend</t>
+          <t>Graphic Designer - Intern</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:44.845632+00:00</t>
+          <t>2026-07-27T16:30:31.543915+00:00</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SDE - Backend - Intern</t>
+          <t>Business Development Specialist (Outbound- International)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Cloudsek</t>
+          <t>Tide</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/cloudsek/jobs/5766402004</t>
+          <t>https://job-boards.greenhouse.io/tide/jobs/7081017003</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>SDE - Backend - Intern</t>
+          <t>Business Development Specialist (Outbound- International)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:42.382537+00:00</t>
+          <t>2026-07-27T16:30:28.879852+00:00</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Business Development Representative Intern - Canada</t>
+          <t>Business Development Specialist (International Sales)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Cloudsek</t>
+          <t>Tide</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/cloudsek/jobs/6005469004</t>
+          <t>https://job-boards.greenhouse.io/tide/jobs/7598880003</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Business Development Representative Intern - Canada</t>
+          <t>Business Development Specialist (International Sales)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:25.892883+00:00</t>
+          <t>2026-07-27T16:30:17.721593+00:00</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>DS/ML Intern</t>
+          <t>Risk Intern - 6 Month Internship Opportunity</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Epifi</t>
+          <t>Towerresearchcapital</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/epifi/08fc1577-4593-4b94-b66b-08e638d29f37</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=7789933</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>A builder mindset is the core of this role and where you'll spend most of your time. But we're a small team building a whole product, not a research lab. The best person here treats ML systems as their primary craft while staying willing to do whatever the product needs — thinking through the product itself, shipping backend or frontend code, untangling data pipelines. We're looking for someone energized by the breadth, not someone who wants to stay in their lane. What you'll work on Evaluation systems for AI features Help build the eval backbone our AI features ship against — failure taxonomies, LLM-as-judge rubrics, golden datasets, calibration against human judgment. Learn what it takes to keep automated scores honest as models and prompts change. A feature with no eval has no quality floor. Model routing &amp; inference economics Get hands-on with how we route work across models — balancing cost, quality, and latency per task. Help run the experiments that justify those choices and catch regressions. Scoring, measurement &amp; signal quality Work on turning noisy, real-world signals into scores you can actually trust — grounded in real statistical rigor, not vibes. Help move heuristic-</t>
+          <t>Risk Intern - 6 Month Internship Opportunity</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:22.213288+00:00</t>
+          <t>2026-07-27T16:30:10.248679+00:00</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Ai Engg Intern</t>
+          <t>Quantitative Trader Intern - Summer 2027</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Epifi</t>
+          <t>Towerresearchcapital</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/epifi/08c743e8-2b29-4f78-827e-5bd90476ed86</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8024128</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Ai Engg Intern</t>
+          <t>Quantitative Trader Intern - Summer 2027</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:12.993097+00:00</t>
+          <t>2026-07-27T16:30:07.980596+00:00</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>[Tech Cooperative Internship 2026] Software Engineer in Back End intern (6 months)</t>
+          <t>Quantitative Trader Intern, PhD</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>Towerresearchcapital</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2189,29 +2233,29 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/agoda/jobs/5443559</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8024138</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>[Tech Cooperative Internship 2026] Software Engineer in Back End intern (6 months)</t>
+          <t>Quantitative Trader Intern, PhD</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-27T16:28:57.849831+00:00</t>
+          <t>2026-07-27T16:30:05.838281+00:00</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>International Payroll Partner</t>
+          <t>Quantitative Developer Intern - Summer 2027</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>Towerresearchcapital</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2223,29 +2267,29 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/agoda/jobs/8063978</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8044334</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>International Payroll Partner</t>
+          <t>Quantitative Developer Intern - Summer 2027</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-27T16:28:36.025672+00:00</t>
+          <t>2026-07-27T16:30:03.426202+00:00</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>GenAI Product Builder Intern</t>
+          <t>Business Analytics Intern - 6 Month Internship Opportunity</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Epifi</t>
+          <t>Towerresearchcapital</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2257,165 +2301,165 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/epifi/4f5b7548-ea0a-4be0-816b-11d712853169</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8041512</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>GenAI Product Builder Intern About us Tetriz is an AI Engineering Intelligence platform that helps engineering organizations become AI-native, faster. We measure how AI coding tools like Cursor, Claude Code, and GitHub Copilot are actually used, improve engineer effectiveness through prompt and workflow coaching, and help engineering leaders demonstrate AI ROI with board-ready, defensible insights. Who should apply This is not a general internship, you should apply only if: - You’ve built or designed things outside of college - You have a portfolio / GitHub of real work - Your work shows initiative, not just completion - You care about problems, not just tools If your experience is mostly coursework, this won’t be a fit. What you’ll get - Work on a real AI product used by engineering teams - Own problems end-to-end, not assist someone else - Exposure to cutting-edge GenAI workflows - A steep learning curve — we’ll push you hard and help you grow fast If you’re hungry and serious, you’ll leave this internship 10x better and ready for the AI-first world. What you’ll do - Build features end-to-end — from idea to production - Work with LLMs, APIs, and internal systems - Create tools th</t>
+          <t>Business Analytics Intern - 6 Month Internship Opportunity</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-27T10:49:04.274532+00:00</t>
+          <t>2026-07-27T16:30:01.432263+00:00</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Copy Writer - Intern</t>
+          <t>Sales Development Representative Intern (Hybrid)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Knowbe4</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774341101</t>
+          <t>https://job-boards.greenhouse.io/knowbe4/jobs/8566454002</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Copy Writer - Intern</t>
+          <t>Sales Development Representative Intern (Hybrid)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-27T10:49:00.838626+00:00</t>
+          <t>2026-07-27T16:29:59.490728+00:00</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Video Editor Intern</t>
+          <t>Sales Development Representative Intern (Hybrid)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Knowbe4</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4771440101</t>
+          <t>https://job-boards.greenhouse.io/knowbe4/jobs/8566457002</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Video Editor Intern</t>
+          <t>Sales Development Representative Intern (Hybrid)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-27T10:48:58.630946+00:00</t>
+          <t>2026-07-27T16:29:55.183092+00:00</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Internship - Content </t>
+          <t>Intern - Industrial Trainee</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Inmobi</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4819749101</t>
+          <t>https://job-boards.greenhouse.io/inmobi/jobs/8029868</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Internship - Content</t>
+          <t>Intern - Industrial Trainee</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-27T10:48:56.06648+00:00</t>
+          <t>2026-07-27T16:29:52.581754+00:00</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Graphic Designer - Intern</t>
+          <t>Intern - Industrial Trainee</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Inmobi</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774342101</t>
+          <t>https://job-boards.greenhouse.io/inmobi/jobs/7793050</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Graphic Designer - Intern</t>
+          <t>Intern - Industrial Trainee</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-27T10:42:53.996409+00:00</t>
+          <t>2026-07-27T16:29:48.780995+00:00</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Copy Writer - Intern</t>
+          <t>Security Consultant Intern</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Cloudsek</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2427,97 +2471,97 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774341101</t>
+          <t>https://job-boards.greenhouse.io/cloudsek/jobs/6115382004</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Copy Writer - Intern</t>
+          <t>Security Consultant Intern</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-27T10:42:50.938109+00:00</t>
+          <t>2026-07-27T16:29:47.193044+00:00</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Graphic Designer - Intern</t>
+          <t xml:space="preserve">SDE Intern - Frontend   </t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Cloudsek</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774342101</t>
+          <t>https://job-boards.greenhouse.io/cloudsek/jobs/5831215004</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Graphic Designer - Intern</t>
+          <t>SDE Intern - Frontend</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-27T10:42:47.32783+00:00</t>
+          <t>2026-07-27T16:29:44.845632+00:00</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Internship - Content </t>
+          <t>SDE - Backend - Intern</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Cloudsek</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4819749101</t>
+          <t>https://job-boards.greenhouse.io/cloudsek/jobs/5766402004</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Internship - Content</t>
+          <t>SDE - Backend - Intern</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-27T10:42:43.192382+00:00</t>
+          <t>2026-07-27T16:29:42.382537+00:00</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Video Editor Intern</t>
+          <t>Business Development Representative Intern - Canada</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Cloudsek</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2529,135 +2573,131 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4771440101</t>
+          <t>https://job-boards.greenhouse.io/cloudsek/jobs/6005469004</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Video Editor Intern</t>
+          <t>Business Development Representative Intern - Canada</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-26T19:14:17.297621+00:00</t>
+          <t>2026-07-27T16:29:25.892883+00:00</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ReactJS Internship</t>
+          <t>DS/ML Intern</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ElevateHQ</t>
+          <t>Epifi</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>₹240000 - ₹420000</t>
-        </is>
-      </c>
+          <t>Data / AI</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/details/4794473734?utm_medium=api&amp;utm_source=e044e1cb</t>
+          <t>https://jobs.lever.co/epifi/08fc1577-4593-4b94-b66b-08e638d29f37</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Position Overview: We are seeking a talented and motivated ReactJS Intern to join our team for a 6-month full-time internship. This is a fantastic opportunity for someone with prior internship experience to deepen their knowledge and skills in ReactJS while working on cutting-edge projects. Responsibilities: Collaborate with the development team to design, develop, and maintain web applications using ReactJS. Write clean, maintainable, and efficient code. Participate in code reviews and contrib…</t>
+          <t>A builder mindset is the core of this role and where you'll spend most of your time. But we're a small team building a whole product, not a research lab. The best person here treats ML systems as their primary craft while staying willing to do whatever the product needs — thinking through the product itself, shipping backend or frontend code, untangling data pipelines. We're looking for someone energized by the breadth, not someone who wants to stay in their lane. What you'll work on Evaluation systems for AI features Help build the eval backbone our AI features ship against — failure taxonomies, LLM-as-judge rubrics, golden datasets, calibration against human judgment. Learn what it takes to keep automated scores honest as models and prompts change. A feature with no eval has no quality floor. Model routing &amp; inference economics Get hands-on with how we route work across models — balancing cost, quality, and latency per task. Help run the experiments that justify those choices and catch regressions. Scoring, measurement &amp; signal quality Work on turning noisy, real-world signals into scores you can actually trust — grounded in real statistical rigor, not vibes. Help move heuristic-</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-26T19:14:13.725695+00:00</t>
+          <t>2026-07-27T16:29:22.213288+00:00</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Developer Internship</t>
+          <t>Ai Engg Intern</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>PBL India</t>
+          <t>Epifi</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/details/4801600698?utm_medium=api&amp;utm_source=e044e1cb</t>
+          <t>https://jobs.lever.co/epifi/08c743e8-2b29-4f78-827e-5bd90476ed86</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Percpktika Brand Lab is a Product Development startup which supports and develops products guiding social innovation. We are looking for smart and talented interns who are capable of working from Delhi or remote and submitting results. At PBL we have an efficient training process which provides resources to grow and nurture your talent. The selected intern(s) will work on following during the internship: 1. Code Reviews and Research. 2. Creating Core features using Node.js and Native Script sup…</t>
+          <t>Ai Engg Intern</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-26T19:14:07.63634+00:00</t>
+          <t>2026-07-27T16:29:12.993097+00:00</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Design Internship</t>
+          <t>[Tech Cooperative Internship 2026] Software Engineer in Back End intern (6 months)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>PBL India</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/details/4801437257?utm_medium=api&amp;utm_source=e044e1cb</t>
+          <t>https://job-boards.greenhouse.io/agoda/jobs/5443559</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Percpktika Brand Lab is a Product Development startup which supports and develops products guiding social innovation. We are looking for smart and talented interns who are capable of working from Delhi or remote and submitting results. At PBL we have an efficient training process which provides resources to grow and nurture your talent. The selected intern(s) will work on following during the internship: 1. Designing User Interface. 2. Experience planning and flow. 3. Product Branding and Desig…</t>
+          <t>[Tech Cooperative Internship 2026] Software Engineer in Back End intern (6 months)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-26T19:13:19.489348+00:00</t>
+          <t>2026-07-27T16:28:57.849831+00:00</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Customer Care Intern</t>
+          <t>International Payroll Partner</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Criteo</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2669,267 +2709,267 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5790410523?se=rFvE0iWJ8RGGXqQIyNVN5Q&amp;utm_medium=api&amp;utm_source=e044e1cb&amp;v=5E72C4726A0DF728D03FF51102E0532CA986DDEA</t>
+          <t>https://job-boards.greenhouse.io/agoda/jobs/8063978</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>This job is with Criteo, an inclusive employer and a member of myGwork – the largest global platform for the LGBTQ business community. Please do not contact the recruiter directly. What You'll Do: The multinational Global Customer Care Team is the first point of contact for Criteo Customers; our goal is to provide excellent customer support to all incoming client requests using email or live chat. We excel at collaboration, communication, and teamwork, as they are key to solving our client's re…</t>
+          <t>International Payroll Partner</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-26T19:13:17.765892+00:00</t>
+          <t>2026-07-27T16:28:36.025672+00:00</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Sales &amp; Strategy Intern</t>
+          <t>GenAI Product Builder Intern</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Criteo</t>
+          <t>Epifi</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5806276940?se=rFvE0iWJ8RGGXqQIyNVN5Q&amp;utm_medium=api&amp;utm_source=e044e1cb&amp;v=B2147145725F724ABD3B0362E330EB1DD5EB962B</t>
+          <t>https://jobs.lever.co/epifi/4f5b7548-ea0a-4be0-816b-11d712853169</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>This job is with Criteo, an inclusive employer and a member of myGwork – the largest global platform for the LGBTQ business community. Please do not contact the recruiter directly. What You'll Do: As a Sales &amp; Strategy Intern, you will be part of our India team that works with new and existing clients. You will be learning and working with brands, analyzing and optimizing campaigns, along with cultivating a strong and productive relationship with clients. This is a 12-month paid, full-time inte…</t>
+          <t>GenAI Product Builder Intern About us Tetriz is an AI Engineering Intelligence platform that helps engineering organizations become AI-native, faster. We measure how AI coding tools like Cursor, Claude Code, and GitHub Copilot are actually used, improve engineer effectiveness through prompt and workflow coaching, and help engineering leaders demonstrate AI ROI with board-ready, defensible insights. Who should apply This is not a general internship, you should apply only if: - You’ve built or designed things outside of college - You have a portfolio / GitHub of real work - Your work shows initiative, not just completion - You care about problems, not just tools If your experience is mostly coursework, this won’t be a fit. What you’ll get - Work on a real AI product used by engineering teams - Own problems end-to-end, not assist someone else - Exposure to cutting-edge GenAI workflows - A steep learning curve — we’ll push you hard and help you grow fast If you’re hungry and serious, you’ll leave this internship 10x better and ready for the AI-first world. What you’ll do - Build features end-to-end — from idea to production - Work with LLMs, APIs, and internal systems - Create tools th</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-26T18:23:56.921677+00:00</t>
+          <t>2026-07-27T10:49:04.274532+00:00</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>GRAPHIC DESIGNER</t>
+          <t>Copy Writer - Intern</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>NEW VINE LIMITED</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-graphic-designer-new-vine-limited-1135316</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774341101</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Graphic Designer (part-time) An exciting opportunity has arisen for a Graphic Designer (part-time) to join us, working remotely with great benefits. The role will work primarily on our books, subscription materials, and digital resources, creating eye-catching covers, inside layouts, and ebooks. Prior experience of working on these types of resources in Adobe Creative Suite is essential, as is a solid understanding of design, layout, typography, and brand. Salary: Â£16,500 (Â£27,500 FTE) Applications close: 29 August 2026 Download the job information (.pdf) Download the application form (.docx) We welcome applicants from all backgrounds and communities, in particular those that are currently under-represented within our staff team. This includes, but is not limited to, people from Black, Asian, and other ethnic groups, especially within our leadership roles. Please mention the word **PROLIFIC** and tag RMjAyLjY2LjE2NC42 when applying to show you read the job post completely (#RMjAyLjY2LjE2NC42). This is a beta feature to avoid spam applicants. Companies can search these words to find applicants that read this and see they're human.</t>
+          <t>Copy Writer - Intern</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-26T18:23:39.597545+00:00</t>
+          <t>2026-07-27T10:49:00.838626+00:00</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Executive Assistant</t>
+          <t>Video Editor Intern</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Ritual AdsÂ®</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-executive-assistant-ritual-adsr-1135344</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4771440101</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Company Description Ritual AdsÂ® is a cutting-edge AI software company that uses generative AI to create tailored, data-driven advertising content on demand. The platform helps organizations quickly produce high-impact, customized ads that align with their brand and audience. By combining advanced machine learning with real-time data, Ritual AdsÂ® aims to improve campaign performance and efficiency. Team members collaborate in a technology-forward environment focused on innovation, scalability, and measurable results. Role Description The Executive Assistant at Ritual AdsÂ® is a full-time, remote role responsible for providing comprehensive administrative and organizational support to company leadership. Day-to-day tasks include managing calendars, scheduling meetings, coordinating travel, and preparing agendas and meeting materials. The Executive Assistant will handle expense reports, track reimbursements, and maintain accurate documentation. The role also includes managing correspondence, drafting and editing communications, organizing digital files, and supporting special projects and operational tasks to ensure smooth executive workflows. Qualifications Strong Executive Adminis</t>
+          <t>Video Editor Intern</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-26T18:23:35.307873+00:00</t>
+          <t>2026-07-27T10:48:58.630946+00:00</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Product Designer</t>
+          <t xml:space="preserve">Internship - Content </t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-product-designer-flint-1135340</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4819749101</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Compensation: $160kâ190k base + meaningful equity About Flint The best education anyone has ever received is one person paying close attention to one student: moving at their pace, noticing what they missed, asking the next question at the right moment. But the current system is built around a compromise with one teacher managing thirty students. Flint exists to take that compromise off the table. Personalized learning, at the scale of a whole school â every student working with something closer to a tutor, and every teacher able to see what's actually happening across their class instead of guessing. Go look at the product before you read any further: app.flintk12.com The Role Students want something that stays with them, going at their pace and helps them get unstuck without just handing over the answer. Teachers want that happening inside a class they still control, and they'd like their evenings back. Admins want proof that the platform they rolled out is leading to teacher productivity and student progress. Your job is to dive deep into this design problem, holding three sets of needs within one product. Weâll trust you to ship designs that are the best possible solution</t>
+          <t>Internship - Content</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-26T18:23:18.030686+00:00</t>
+          <t>2026-07-27T10:48:56.06648+00:00</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Join our UK team</t>
+          <t>Graphic Designer - Intern</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Workdry Germany</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-join-our-uk-team-workdry-germany-1135314</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774342101</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>BracknellPump Rental SolutionsBracknellPump Rental SolutionsGreat YarmouthPump Rental SolutionsNottinghamPump Rental SolutionsAberdeenPump Rental SolutionsConwyPump Rental SolutionsStokeWorkdry - Group Central ServicesStokeWorkdry - Group Central ServicesWorkingtonPump Rental Solutions Please mention the word **GREATNESS** and tag RMjAyLjY2LjE2NC42 when applying to show you read the job post completely (#RMjAyLjY2LjE2NC42). This is a beta feature to avoid spam applicants. Companies can search these words to find applicants that read this and see they're human.</t>
+          <t>Graphic Designer - Intern</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-26T18:23:11.834056+00:00</t>
+          <t>2026-07-27T10:42:53.996409+00:00</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Safety Data Analyst</t>
+          <t>Copy Writer - Intern</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SkyWest Airlines</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-safety-data-analyst-skywest-airlines-1135445</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774341101</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>About SkyWest With over 16,000 aviation professionals operating thousands of daily flights, SkyWest Airlines connects millions of passengers each month to hundreds of destinations across North America. SkyWest operates in partnership with Delta Air Lines, United Airlines, American Airlines, and Alaska Airlines and has a fleet of nearly 450 aircraft. Headquartered in St. George, Utah, SkyWest's industry-leading workforce and excellent leadership team have consistently generated solid operational and economic performance, setting the standard for excellence in the regional industry. SkyWest employees enjoy a distinctive and unmatched culture of teamwork, respect, quality, and professionalism, along with world-class benefits such as a 401(k) match, Performance Rewards, health care, retirement, and discounted travel worldwide. Primary Job Duties Analyze, compile, and report safety data to support all SkyWest safety programs. Collect, analyze, and report safety assurance data from multiple safety data sources. Identify, monitor, and communicate safety performance trends and emerging risks. Track, maintain, and report key performance indicators (KPIs) for the Safety Department, including</t>
+          <t>Copy Writer - Intern</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-26T18:22:46.777033+00:00</t>
+          <t>2026-07-27T10:42:50.938109+00:00</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Engineering Manager - Edge AI</t>
+          <t>Graphic Designer - Intern</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SumUp</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sumup/engineering-manager-edge-ai-berlin-258996</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774342101</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Our AI Platform &amp;amp; Edge team sits at the heart of how SumUp is scaling intelligent, merchant-facing experiences across millions of interactions. We build and operate the AI systems — from LLM-powered assistants to agentic platforms — that directly shape how merchants get support, resolve issues, and engage with SumUp's products. As Engineering Manager for Edge, you'll take ownership of a growing, cross-functional team of engineers and ML specialists, leading the execution of some of our most technically complex and commercially critical AI initiatives. This is a rare opportunity to lead meaningful AI work at scale — not just shipping features, but shaping how an entire platform evolves. What you'll do Lead the day-to-day execution of the Edge AI team, translating long-term product vision into clear sprint roadmaps and measurable delivery milestones Own the migration of our AI assistant to an autonomous agentic setup, maintaining performance while expanding AI support across all merchant-facing channels Set the technical direction for LLM-powered system design, making clear tradeoffs across quality, latency, and cost Build a data-informed engineering culture by defining performan</t>
+          <t>Graphic Designer - Intern</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-26T18:22:37.744444+00:00</t>
+          <t>2026-07-27T10:42:47.32783+00:00</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Chief Marketing Officer (m/w/d)</t>
+          <t xml:space="preserve">Internship - Content </t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>InkuPlay UG (haftungsbeschränkt)</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2941,184 +2981,630 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/inkuplay-ug-haftungsbeschrankt/chief-marketing-officer-biesenthal-255944</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4819749101</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>InkuPlay ist ein wachstumsorientiertes Unternehmen aus dem Gaming- und E-Sports-Umfeld. Wir entwickeln Marken, Communities, digitale Formate und Partnerschaften an der Schnittstelle von Gaming, Entertainment, Content, Creator Economy und E-Sports. Unser Ziel ist es, InkuPlay als moderne, international relevante Gaming- und E-Sports-Marke zu etablieren. Dafür suchen wir eine unternehmerisch denkende Führungspersönlichkeit, die unsere Marketingstrategie entwickelt, unsere Markenpositionierung schärft und nachhaltiges Wachstum vorantreibt. Als Chief Marketing Officer (m/w/d) übernimmst du die Gesamtverantwortung für Marketing, Marke, Kommunikation und Wachstum bei InkuPlay. Du entwickelst nicht nur Kampagnen, sondern baust gemeinsam mit der Geschäftsführung eine belastbare Marketingorganisation auf. Dabei verbindest du strategische Markenführung mit datengetriebenem Growth Marketing, aufmerksamkeitsstarkem Content und kommerziell erfolgreichen Partnerschaften. Du berichtest direkt an den Founder &amp;#x26; CEO und arbeitest eng mit den Bereichen Esports, Content &amp;#x26; Media, Partnerships, Sales, Community, Recruiting und Business Development zusammen. Aufgaben Marketing- und Unternehmens</t>
+          <t>Internship - Content</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-26T18:22:34.380054+00:00</t>
+          <t>2026-07-27T10:42:43.192382+00:00</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Head of People &amp; Culture / HR (m/w/d)</t>
+          <t>Video Editor Intern</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>InkuPlay UG (haftungsbeschränkt)</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/inkuplay-ug-haftungsbeschrankt/head-of-people-culture-hr-biesenthal-163623</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4771440101</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t xml:space="preserve">InkuPlay ist ein wachsendes Unternehmen aus den Bereichen Gaming, Esports, digitale Plattformen, Content, Community und Partnerschaften. Wir befinden uns in einer Phase des strukturellen Aufbaus und der Professionalisierung. Dafür suchen wir eine erfahrene Persönlichkeit, die unsere Personalorganisation nicht nur verwaltet, sondern aktiv gestaltet. Als Head of People &amp;#x26; Culture / HR übernimmst du die Verantwortung für den Aufbau moderner, rechtssicherer und skalierbarer Personalstrukturen. Du arbeitest eng mit dem Founder &amp;#x26; CEO, dem operativen Management, den Führungskräften sowie externen arbeitsrechtlichen und steuerlichen Beratern zusammen. Die Position verbindet strategische Personalarbeit mit operativer Umsetzung. Gesucht wird daher keine rein beratende HR-Funktion, sondern eine Person, die Verantwortung übernimmt, Entscheidungen vorbereitet, Prozesse etabliert und Themen zuverlässig bis zum Abschluss begleitet. Deine Rolle Als Head of People &amp;#x26; Culture / HR verantwortest du sämtliche personalbezogenen Themen bei InkuPlay. Du entwickelst eine professionelle HR-Struktur, die zu einem dynamischen Startup im Gaming- und Esports-Umfeld passt. Dabei stellst du sicher, </t>
+          <t>Video Editor Intern</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-26T18:22:32.624515+00:00</t>
+          <t>2026-07-26T19:14:17.297621+00:00</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>ReactJS Internship</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>ElevateHQ</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr"/>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>₹240000 - ₹420000</t>
+        </is>
+      </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sayano-deutschland-gmbh/praktikum-amazon-ppc-performance-marketing-im-e-commerce-start-up-stuttgart-189082</t>
+          <t>https://www.adzuna.in/details/4794473734?utm_medium=api&amp;utm_source=e044e1cb</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Du willst mitgestalten statt nur zuschauen? Dann bist Du bei uns richtig. Wir sind Sayano – ein modernes, international tätiges E-Commerce-Unternehmen hinter Marken wie MIAMIO, Tortillada und Calmado. Unsere Produkte erreichen Kundinnen und Kunden in mehr als 80 Ländern. Die Financial Times hat uns vier Jahre in Folge als eines der am schnellsten wachsenden Unternehmen Europas ausgezeichnet. Wir arbeiten schnell, datengetrieben und konsequent mit modernen KI-Technologien. KI ist für uns kein Zukunftsthema, sondern fester Bestandteil unseres Arbeitsalltags – von Analysen und Recherchen über Automatisierungen bis zur Optimierung unserer Werbekampagnen. Aufgaben Du unterstützt bei der Analyse und Optimierung unserer Amazon-PPC-Kampagnen Du arbeitest mit Sponsored Products, Sponsored Brands und Sponsored Display Du führst Keyword-, Suchbegriff- und Wettbewerbsanalysen durch Du identifizierst profitable Suchbegriffe und entwickelst diese gemeinsam mit uns weiter Du hilfst dabei, unnötige Werbeausgaben zu erkennen und zu reduzieren Du unterstützt bei der Optimierung von Geboten, Budgets, Platzierungen und negativen Keywords Du analysierst Kennzahlen wie ACOS, TACOS, ROAS, CPC, CTR und Co</t>
+          <t>Position Overview: We are seeking a talented and motivated ReactJS Intern to join our team for a 6-month full-time internship. This is a fantastic opportunity for someone with prior internship experience to deepen their knowledge and skills in ReactJS while working on cutting-edge projects. Responsibilities: Collaborate with the development team to design, develop, and maintain web applications using ReactJS. Write clean, maintainable, and efficient code. Participate in code reviews and contrib…</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-26T18:22:28.361273+00:00</t>
+          <t>2026-07-26T19:14:13.725695+00:00</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Brand &amp; Content Lead</t>
+          <t>Developer Internship</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Klar</t>
+          <t>PBL India</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/klar/brand-content-lead-munich-463374</t>
+          <t>https://www.adzuna.in/details/4801600698?utm_medium=api&amp;utm_source=e044e1cb</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>In Short: We are looking for someone that loves content and eCommerce to own our entire brand surface — content, community, product marketing, and website — and turn Klar into the go-to resource for actionable eCom knowledge in Europe. About Klar 🚀 The Mission Klar is the Data Operating System for growing eCommerce companies, meaning no more spreadsheets . We integrate with all of a brand's data sources to provide a holistic understanding of their business, offering detailed insights on how to accelerate growth and increase profitability. 🛍️ The Reach We are already the "single source of truth" for over 1,000 leading eCom brands. Market leaders like Sunday Natural, Loop Earplugs, Holy, Maniko, and Armed Angels use Klar to make better decisions every single day. 🤝 The Backstory We deeply empathize with our customers because we were our customers. The founders (who met in South Africa working for Zando) spent the last 10 years in e-commerce. We know the pain of running these businesses, and we built Klar specifically to solve it. ✨ The Principle Our guiding principle is Do Work You Are Proud Of . We emphasize long-term quality over short-term results. We evaluate our tools and dec</t>
+          <t>Percpktika Brand Lab is a Product Development startup which supports and develops products guiding social innovation. We are looking for smart and talented interns who are capable of working from Delhi or remote and submitting results. At PBL we have an efficient training process which provides resources to grow and nurture your talent. The selected intern(s) will work on following during the internship: 1. Code Reviews and Research. 2. Creating Core features using Node.js and Native Script sup…</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-26T18:22:23.542927+00:00</t>
+          <t>2026-07-26T19:14:07.63634+00:00</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Kreativer Allrounder Marketing (m/w/d) | Gestalte unseren Markenauftritt aktiv</t>
+          <t>Design Internship</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Autohaus Wernsing GmbH</t>
+          <t>PBL India</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autohaus-wernsing-gmbh/kreativer-allrounder-marketing-gestalte-unseren-markenauftritt-aktiv-bersenbruck-288838</t>
+          <t>https://www.adzuna.in/details/4801437257?utm_medium=api&amp;utm_source=e044e1cb</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Werde kreativ. Mach unsere Marken sichtbar. Du hast Freude an Social Media, Content Creation und kreativem Marketing? Du möchtest nicht einfach nur bestehende Aufgaben abarbeiten, sondern einen Marketingbereich aktiv mitgestalten und weiterentwickeln? Dann bist du bei uns genau richtig! Für unsere Unternehmen Autohaus Wernsing und 2Rad Wernsing suchen wir eine kreative und engagierte Persönlichkeit, die unseren Außenauftritt eigenverantwortlich weiterentwickelt und gemeinsam mit der Geschäftsführung den Marketingbereich aufbaut. Du arbeitest auf Basis unseres bestehenden Markenbooks mit klar definiertem Corporate Design und hast gleichzeitig viel Freiraum für eigene Ideen und kreative Konzepte. Der Schwerpunkt deiner Tätigkeit liegt eindeutig im Marketing. Ein kleiner Teil deiner Arbeitszeit unterstützt unser Team bei Veranstaltungen oder vertriebsnahen Projekten. Ob in Teilzeit oder auf geringfügiger Basis – wir sind flexibel. Ein Teil deiner Arbeit kann nach Absprache auch im Homeoffice erledigt werden. Aufgaben Marketing &amp;#x26; Content Creation Eigenverantwortlicher Aufbau und Weiterentwicklung unseres Marketingbereichs in enger Abstimmung mit der Geschäftsführung Planung, Erste</t>
+          <t>Percpktika Brand Lab is a Product Development startup which supports and develops products guiding social innovation. We are looking for smart and talented interns who are capable of working from Delhi or remote and submitting results. At PBL we have an efficient training process which provides resources to grow and nurture your talent. The selected intern(s) will work on following during the internship: 1. Designing User Interface. 2. Experience planning and flow. 3. Product Branding and Desig…</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-17T10:23:01.374271+00:00</t>
+          <t>2026-07-26T19:13:19.489348+00:00</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Test Internship</t>
+          <t>Customer Care Intern</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Test Company</t>
+          <t>Criteo</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>10,000/mo</t>
-        </is>
-      </c>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
+          <t>https://www.adzuna.in/land/ad/5790410523?se=rFvE0iWJ8RGGXqQIyNVN5Q&amp;utm_medium=api&amp;utm_source=e044e1cb&amp;v=5E72C4726A0DF728D03FF51102E0532CA986DDEA</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>This job is with Criteo, an inclusive employer and a member of myGwork – the largest global platform for the LGBTQ business community. Please do not contact the recruiter directly. What You'll Do: The multinational Global Customer Care Team is the first point of contact for Criteo Customers; our goal is to provide excellent customer support to all incoming client requests using email or live chat. We excel at collaboration, communication, and teamwork, as they are key to solving our client's re…</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-07-26T19:13:17.765892+00:00</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Sales &amp; Strategy Intern</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Criteo</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5806276940?se=rFvE0iWJ8RGGXqQIyNVN5Q&amp;utm_medium=api&amp;utm_source=e044e1cb&amp;v=B2147145725F724ABD3B0362E330EB1DD5EB962B</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>This job is with Criteo, an inclusive employer and a member of myGwork – the largest global platform for the LGBTQ business community. Please do not contact the recruiter directly. What You'll Do: As a Sales &amp; Strategy Intern, you will be part of our India team that works with new and existing clients. You will be learning and working with brands, analyzing and optimizing campaigns, along with cultivating a strong and productive relationship with clients. This is a 12-month paid, full-time inte…</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:23:56.921677+00:00</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>GRAPHIC DESIGNER</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>NEW VINE LIMITED</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-graphic-designer-new-vine-limited-1135316</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Graphic Designer (part-time) An exciting opportunity has arisen for a Graphic Designer (part-time) to join us, working remotely with great benefits. The role will work primarily on our books, subscription materials, and digital resources, creating eye-catching covers, inside layouts, and ebooks. Prior experience of working on these types of resources in Adobe Creative Suite is essential, as is a solid understanding of design, layout, typography, and brand. Salary: Â£16,500 (Â£27,500 FTE) Applications close: 29 August 2026 Download the job information (.pdf) Download the application form (.docx) We welcome applicants from all backgrounds and communities, in particular those that are currently under-represented within our staff team. This includes, but is not limited to, people from Black, Asian, and other ethnic groups, especially within our leadership roles. Please mention the word **PROLIFIC** and tag RMjAyLjY2LjE2NC42 when applying to show you read the job post completely (#RMjAyLjY2LjE2NC42). This is a beta feature to avoid spam applicants. Companies can search these words to find applicants that read this and see they're human.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:23:39.597545+00:00</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Executive Assistant</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Ritual AdsÂ®</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-executive-assistant-ritual-adsr-1135344</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Company Description Ritual AdsÂ® is a cutting-edge AI software company that uses generative AI to create tailored, data-driven advertising content on demand. The platform helps organizations quickly produce high-impact, customized ads that align with their brand and audience. By combining advanced machine learning with real-time data, Ritual AdsÂ® aims to improve campaign performance and efficiency. Team members collaborate in a technology-forward environment focused on innovation, scalability, and measurable results. Role Description The Executive Assistant at Ritual AdsÂ® is a full-time, remote role responsible for providing comprehensive administrative and organizational support to company leadership. Day-to-day tasks include managing calendars, scheduling meetings, coordinating travel, and preparing agendas and meeting materials. The Executive Assistant will handle expense reports, track reimbursements, and maintain accurate documentation. The role also includes managing correspondence, drafting and editing communications, organizing digital files, and supporting special projects and operational tasks to ensure smooth executive workflows. Qualifications Strong Executive Adminis</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:23:35.307873+00:00</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Product Designer</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Flint</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-product-designer-flint-1135340</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Compensation: $160kâ190k base + meaningful equity About Flint The best education anyone has ever received is one person paying close attention to one student: moving at their pace, noticing what they missed, asking the next question at the right moment. But the current system is built around a compromise with one teacher managing thirty students. Flint exists to take that compromise off the table. Personalized learning, at the scale of a whole school â every student working with something closer to a tutor, and every teacher able to see what's actually happening across their class instead of guessing. Go look at the product before you read any further: app.flintk12.com The Role Students want something that stays with them, going at their pace and helps them get unstuck without just handing over the answer. Teachers want that happening inside a class they still control, and they'd like their evenings back. Admins want proof that the platform they rolled out is leading to teacher productivity and student progress. Your job is to dive deep into this design problem, holding three sets of needs within one product. Weâll trust you to ship designs that are the best possible solution</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:23:18.030686+00:00</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Join our UK team</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Workdry Germany</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-join-our-uk-team-workdry-germany-1135314</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>BracknellPump Rental SolutionsBracknellPump Rental SolutionsGreat YarmouthPump Rental SolutionsNottinghamPump Rental SolutionsAberdeenPump Rental SolutionsConwyPump Rental SolutionsStokeWorkdry - Group Central ServicesStokeWorkdry - Group Central ServicesWorkingtonPump Rental Solutions Please mention the word **GREATNESS** and tag RMjAyLjY2LjE2NC42 when applying to show you read the job post completely (#RMjAyLjY2LjE2NC42). This is a beta feature to avoid spam applicants. Companies can search these words to find applicants that read this and see they're human.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:23:11.834056+00:00</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Safety Data Analyst</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>SkyWest Airlines</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Data / AI</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-safety-data-analyst-skywest-airlines-1135445</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>About SkyWest With over 16,000 aviation professionals operating thousands of daily flights, SkyWest Airlines connects millions of passengers each month to hundreds of destinations across North America. SkyWest operates in partnership with Delta Air Lines, United Airlines, American Airlines, and Alaska Airlines and has a fleet of nearly 450 aircraft. Headquartered in St. George, Utah, SkyWest's industry-leading workforce and excellent leadership team have consistently generated solid operational and economic performance, setting the standard for excellence in the regional industry. SkyWest employees enjoy a distinctive and unmatched culture of teamwork, respect, quality, and professionalism, along with world-class benefits such as a 401(k) match, Performance Rewards, health care, retirement, and discounted travel worldwide. Primary Job Duties Analyze, compile, and report safety data to support all SkyWest safety programs. Collect, analyze, and report safety assurance data from multiple safety data sources. Identify, monitor, and communicate safety performance trends and emerging risks. Track, maintain, and report key performance indicators (KPIs) for the Safety Department, including</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:22:46.777033+00:00</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Engineering Manager - Edge AI</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>SumUp</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Data / AI</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/sumup/engineering-manager-edge-ai-berlin-258996</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Our AI Platform &amp;amp; Edge team sits at the heart of how SumUp is scaling intelligent, merchant-facing experiences across millions of interactions. We build and operate the AI systems — from LLM-powered assistants to agentic platforms — that directly shape how merchants get support, resolve issues, and engage with SumUp's products. As Engineering Manager for Edge, you'll take ownership of a growing, cross-functional team of engineers and ML specialists, leading the execution of some of our most technically complex and commercially critical AI initiatives. This is a rare opportunity to lead meaningful AI work at scale — not just shipping features, but shaping how an entire platform evolves. What you'll do Lead the day-to-day execution of the Edge AI team, translating long-term product vision into clear sprint roadmaps and measurable delivery milestones Own the migration of our AI assistant to an autonomous agentic setup, maintaining performance while expanding AI support across all merchant-facing channels Set the technical direction for LLM-powered system design, making clear tradeoffs across quality, latency, and cost Build a data-informed engineering culture by defining performan</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:22:37.744444+00:00</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Chief Marketing Officer (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>InkuPlay UG (haftungsbeschränkt)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/inkuplay-ug-haftungsbeschrankt/chief-marketing-officer-biesenthal-255944</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>InkuPlay ist ein wachstumsorientiertes Unternehmen aus dem Gaming- und E-Sports-Umfeld. Wir entwickeln Marken, Communities, digitale Formate und Partnerschaften an der Schnittstelle von Gaming, Entertainment, Content, Creator Economy und E-Sports. Unser Ziel ist es, InkuPlay als moderne, international relevante Gaming- und E-Sports-Marke zu etablieren. Dafür suchen wir eine unternehmerisch denkende Führungspersönlichkeit, die unsere Marketingstrategie entwickelt, unsere Markenpositionierung schärft und nachhaltiges Wachstum vorantreibt. Als Chief Marketing Officer (m/w/d) übernimmst du die Gesamtverantwortung für Marketing, Marke, Kommunikation und Wachstum bei InkuPlay. Du entwickelst nicht nur Kampagnen, sondern baust gemeinsam mit der Geschäftsführung eine belastbare Marketingorganisation auf. Dabei verbindest du strategische Markenführung mit datengetriebenem Growth Marketing, aufmerksamkeitsstarkem Content und kommerziell erfolgreichen Partnerschaften. Du berichtest direkt an den Founder &amp;#x26; CEO und arbeitest eng mit den Bereichen Esports, Content &amp;#x26; Media, Partnerships, Sales, Community, Recruiting und Business Development zusammen. Aufgaben Marketing- und Unternehmens</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:22:34.380054+00:00</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Head of People &amp; Culture / HR (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>InkuPlay UG (haftungsbeschränkt)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/inkuplay-ug-haftungsbeschrankt/head-of-people-culture-hr-biesenthal-163623</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">InkuPlay ist ein wachsendes Unternehmen aus den Bereichen Gaming, Esports, digitale Plattformen, Content, Community und Partnerschaften. Wir befinden uns in einer Phase des strukturellen Aufbaus und der Professionalisierung. Dafür suchen wir eine erfahrene Persönlichkeit, die unsere Personalorganisation nicht nur verwaltet, sondern aktiv gestaltet. Als Head of People &amp;#x26; Culture / HR übernimmst du die Verantwortung für den Aufbau moderner, rechtssicherer und skalierbarer Personalstrukturen. Du arbeitest eng mit dem Founder &amp;#x26; CEO, dem operativen Management, den Führungskräften sowie externen arbeitsrechtlichen und steuerlichen Beratern zusammen. Die Position verbindet strategische Personalarbeit mit operativer Umsetzung. Gesucht wird daher keine rein beratende HR-Funktion, sondern eine Person, die Verantwortung übernimmt, Entscheidungen vorbereitet, Prozesse etabliert und Themen zuverlässig bis zum Abschluss begleitet. Deine Rolle Als Head of People &amp;#x26; Culture / HR verantwortest du sämtliche personalbezogenen Themen bei InkuPlay. Du entwickelst eine professionelle HR-Struktur, die zu einem dynamischen Startup im Gaming- und Esports-Umfeld passt. Dabei stellst du sicher, </t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:22:32.624515+00:00</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Sayano Deutschland GmbH</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/sayano-deutschland-gmbh/praktikum-amazon-ppc-performance-marketing-im-e-commerce-start-up-stuttgart-189082</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Du willst mitgestalten statt nur zuschauen? Dann bist Du bei uns richtig. Wir sind Sayano – ein modernes, international tätiges E-Commerce-Unternehmen hinter Marken wie MIAMIO, Tortillada und Calmado. Unsere Produkte erreichen Kundinnen und Kunden in mehr als 80 Ländern. Die Financial Times hat uns vier Jahre in Folge als eines der am schnellsten wachsenden Unternehmen Europas ausgezeichnet. Wir arbeiten schnell, datengetrieben und konsequent mit modernen KI-Technologien. KI ist für uns kein Zukunftsthema, sondern fester Bestandteil unseres Arbeitsalltags – von Analysen und Recherchen über Automatisierungen bis zur Optimierung unserer Werbekampagnen. Aufgaben Du unterstützt bei der Analyse und Optimierung unserer Amazon-PPC-Kampagnen Du arbeitest mit Sponsored Products, Sponsored Brands und Sponsored Display Du führst Keyword-, Suchbegriff- und Wettbewerbsanalysen durch Du identifizierst profitable Suchbegriffe und entwickelst diese gemeinsam mit uns weiter Du hilfst dabei, unnötige Werbeausgaben zu erkennen und zu reduzieren Du unterstützt bei der Optimierung von Geboten, Budgets, Platzierungen und negativen Keywords Du analysierst Kennzahlen wie ACOS, TACOS, ROAS, CPC, CTR und Co</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:22:28.361273+00:00</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Brand &amp; Content Lead</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Klar</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/klar/brand-content-lead-munich-463374</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>In Short: We are looking for someone that loves content and eCommerce to own our entire brand surface — content, community, product marketing, and website — and turn Klar into the go-to resource for actionable eCom knowledge in Europe. About Klar 🚀 The Mission Klar is the Data Operating System for growing eCommerce companies, meaning no more spreadsheets . We integrate with all of a brand's data sources to provide a holistic understanding of their business, offering detailed insights on how to accelerate growth and increase profitability. 🛍️ The Reach We are already the "single source of truth" for over 1,000 leading eCom brands. Market leaders like Sunday Natural, Loop Earplugs, Holy, Maniko, and Armed Angels use Klar to make better decisions every single day. 🤝 The Backstory We deeply empathize with our customers because we were our customers. The founders (who met in South Africa working for Zando) spent the last 10 years in e-commerce. We know the pain of running these businesses, and we built Klar specifically to solve it. ✨ The Principle Our guiding principle is Do Work You Are Proud Of . We emphasize long-term quality over short-term results. We evaluate our tools and dec</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:22:23.542927+00:00</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Kreativer Allrounder Marketing (m/w/d) | Gestalte unseren Markenauftritt aktiv</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Autohaus Wernsing GmbH</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autohaus-wernsing-gmbh/kreativer-allrounder-marketing-gestalte-unseren-markenauftritt-aktiv-bersenbruck-288838</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Werde kreativ. Mach unsere Marken sichtbar. Du hast Freude an Social Media, Content Creation und kreativem Marketing? Du möchtest nicht einfach nur bestehende Aufgaben abarbeiten, sondern einen Marketingbereich aktiv mitgestalten und weiterentwickeln? Dann bist du bei uns genau richtig! Für unsere Unternehmen Autohaus Wernsing und 2Rad Wernsing suchen wir eine kreative und engagierte Persönlichkeit, die unseren Außenauftritt eigenverantwortlich weiterentwickelt und gemeinsam mit der Geschäftsführung den Marketingbereich aufbaut. Du arbeitest auf Basis unseres bestehenden Markenbooks mit klar definiertem Corporate Design und hast gleichzeitig viel Freiraum für eigene Ideen und kreative Konzepte. Der Schwerpunkt deiner Tätigkeit liegt eindeutig im Marketing. Ein kleiner Teil deiner Arbeitszeit unterstützt unser Team bei Veranstaltungen oder vertriebsnahen Projekten. Ob in Teilzeit oder auf geringfügiger Basis – wir sind flexibel. Ein Teil deiner Arbeit kann nach Absprache auch im Homeoffice erledigt werden. Aufgaben Marketing &amp;#x26; Content Creation Eigenverantwortlicher Aufbau und Weiterentwicklung unseres Marketingbereichs in enger Abstimmung mit der Geschäftsführung Planung, Erste</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-07-17T10:23:01.374271+00:00</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Test Internship</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Test Company</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>10,000/mo</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
           <t>https://example.com</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr">
+      <c r="H90" t="inlineStr">
         <is>
           <t>This is a test listing</t>
         </is>

</xml_diff>